<commit_message>
Add Territory tab so reps declare their region (states/areas)
Reps had no place to indicate their geographic domain. Add a Territory
sheet to the intake workbook (rep name, territory label, states covered,
optional sub-state areas, region avg case) and thread it through the
builder: it sets the report title, stamps rep/states/areas into meta and
territory, and drives region_avg_case for the reservoir opportunity math.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GxChwdgepdKhJ25wYKRVB7
</commit_message>
<xml_diff>
--- a/tools/account-cards-alt/territory_template.xlsx
+++ b/tools/account-cards-alt/territory_template.xlsx
@@ -8,10 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="READ ME" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accounts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Surgeons" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referrers" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reservoirs" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Territory" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accounts" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Surgeons" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referrers" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reservoirs" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -158,132 +159,32 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Priority rank (1 = top)</t>
+        <t>Your name — the territory owner</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>e.g. Columbia (NYP)</t>
+        <t>Your territory label, e.g. Northeast / Great Lakes / SoCal</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Short unique code, e.g. CUMC</t>
+        <t>The states/areas you own — semicolon list, e.g. NY;NJ;CT;MA. This is your region: it scopes the claims pull and the facility research.</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>e.g. NewYork-Presbyterian</t>
+        <t>Optional — for split states, name the metros/counties you hold, e.g. NY = NYC metro + Westchester + Long Island</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Installed / Contested / Installing / Pipeline / Competitive</t>
+        <t>Region average revenue per LITT case ($). Blank = 18,300 default.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Your one-line posture, e.g. Expand, priority</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>Semicolon list: NeuroBlate;Visualase;ClearPoint</t>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
-      <text>
-        <t>High / Medium / Long-horizon</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <t>Free-text account narrative</t>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <t>From the robot library, or blank</t>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
-      <text>
-        <t>From the navigation library, or blank</t>
-      </text>
-    </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
-      <text>
-        <t>e.g. iMRI / 3T / blank</t>
-      </text>
-    </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
-      <text>
-        <t>e.g. active / blank</t>
-      </text>
-    </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
-      <text>
-        <t>SEEG claims/volume (number), or 0</t>
-      </text>
-    </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
-      <text>
-        <t>Tumor+epilepsy craniotomies/yr (number)</t>
-      </text>
-    </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
-      <text>
-        <t>Net sales 2024 ($)</t>
-      </text>
-    </comment>
-    <comment ref="Q1" authorId="0" shapeId="0">
-      <text>
-        <t>Net sales 2025 ($)</t>
-      </text>
-    </comment>
-    <comment ref="R1" authorId="0" shapeId="0">
-      <text>
-        <t>Net sales 2026 YTD ($)</t>
-      </text>
-    </comment>
-    <comment ref="S1" authorId="0" shapeId="0">
-      <text>
-        <t>Full-year 2026 projection ($)</t>
-      </text>
-    </comment>
-    <comment ref="T1" authorId="0" shapeId="0">
-      <text>
-        <t>LITT cases logged (3yr)</t>
-      </text>
-    </comment>
-    <comment ref="U1" authorId="0" shapeId="0">
-      <text>
-        <t>Laser probes 2024</t>
-      </text>
-    </comment>
-    <comment ref="V1" authorId="0" shapeId="0">
-      <text>
-        <t>Laser probes 2025</t>
-      </text>
-    </comment>
-    <comment ref="W1" authorId="0" shapeId="0">
-      <text>
-        <t>Laser probes 2026</t>
-      </text>
-    </comment>
-    <comment ref="X1" authorId="0" shapeId="0">
-      <text>
-        <t>Plan's realistic incremental $/yr</t>
-      </text>
-    </comment>
-    <comment ref="Y1" authorId="0" shapeId="0">
-      <text>
-        <t>Plan's incremental cases target</t>
-      </text>
-    </comment>
-    <comment ref="Z1" authorId="0" shapeId="0">
-      <text>
-        <t>Up / Flat / Down / New / Competitive</t>
+        <t>Any territory-level notes</t>
       </text>
     </comment>
   </commentList>
@@ -298,57 +199,132 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Account acronym this surgeon belongs to</t>
+        <t>Priority rank (1 = top)</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Surgeon full name</t>
+        <t>e.g. Columbia (NYP)</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Performer (does LITT) or Target (LITT-naïve)</t>
+        <t>Short unique code, e.g. CUMC</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>LITT cases if a performer, else blank</t>
+        <t>e.g. NewYork-Presbyterian</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>SEEG volume (number)</t>
+        <t>Installed / Contested / Installing / Pipeline / Competitive</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Epilepsy craniotomies (number)</t>
+        <t>Your one-line posture, e.g. Expand, priority</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>Tumor craniotomies (number)</t>
+        <t>Semicolon list: NeuroBlate;Visualase;ClearPoint</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
       <text>
-        <t>Short archetype, e.g. SEEG-driven epilepsy ablation</t>
+        <t>High / Medium / Long-horizon</t>
       </text>
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
-        <t>Y if a LITT KOL</t>
+        <t>Free-text account narrative</t>
       </text>
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
       <text>
-        <t>Optional bio link</t>
+        <t>From the robot library, or blank</t>
       </text>
     </comment>
     <comment ref="K1" authorId="0" shapeId="0">
       <text>
-        <t>Optional PubMed link</t>
+        <t>From the navigation library, or blank</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>e.g. iMRI / 3T / blank</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <t>e.g. active / blank</t>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <t>SEEG claims/volume (number), or 0</t>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0" shapeId="0">
+      <text>
+        <t>Tumor+epilepsy craniotomies/yr (number)</t>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="0" shapeId="0">
+      <text>
+        <t>Net sales 2024 ($)</t>
+      </text>
+    </comment>
+    <comment ref="Q1" authorId="0" shapeId="0">
+      <text>
+        <t>Net sales 2025 ($)</t>
+      </text>
+    </comment>
+    <comment ref="R1" authorId="0" shapeId="0">
+      <text>
+        <t>Net sales 2026 YTD ($)</t>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="0" shapeId="0">
+      <text>
+        <t>Full-year 2026 projection ($)</t>
+      </text>
+    </comment>
+    <comment ref="T1" authorId="0" shapeId="0">
+      <text>
+        <t>LITT cases logged (3yr)</t>
+      </text>
+    </comment>
+    <comment ref="U1" authorId="0" shapeId="0">
+      <text>
+        <t>Laser probes 2024</t>
+      </text>
+    </comment>
+    <comment ref="V1" authorId="0" shapeId="0">
+      <text>
+        <t>Laser probes 2025</t>
+      </text>
+    </comment>
+    <comment ref="W1" authorId="0" shapeId="0">
+      <text>
+        <t>Laser probes 2026</t>
+      </text>
+    </comment>
+    <comment ref="X1" authorId="0" shapeId="0">
+      <text>
+        <t>Plan's realistic incremental $/yr</t>
+      </text>
+    </comment>
+    <comment ref="Y1" authorId="0" shapeId="0">
+      <text>
+        <t>Plan's incremental cases target</t>
+      </text>
+    </comment>
+    <comment ref="Z1" authorId="0" shapeId="0">
+      <text>
+        <t>Up / Flat / Down / New / Competitive</t>
       </text>
     </comment>
   </commentList>
@@ -363,22 +339,57 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Account acronym</t>
+        <t>Account acronym this surgeon belongs to</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Referrer name</t>
+        <t>Surgeon full name</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>e.g. Epilepsy (DRE) / Mets / Rad-necrosis</t>
+        <t>Performer (does LITT) or Target (LITT-naïve)</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Patient pool size OR number of referrals (number)</t>
+        <t>LITT cases if a performer, else blank</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>SEEG volume (number)</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Epilepsy craniotomies (number)</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Tumor craniotomies (number)</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>Short archetype, e.g. SEEG-driven epilepsy ablation</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>Y if a LITT KOL</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional bio link</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional PubMed link</t>
       </text>
     </comment>
   </commentList>
@@ -386,6 +397,36 @@
 </file>
 
 <file path=xl/comments/comment4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>template</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Account acronym</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Referrer name</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>e.g. Epilepsy (DRE) / Mets / Rad-necrosis</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Patient pool size OR number of referrals (number)</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment5.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>template</author>
@@ -704,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -723,53 +764,60 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>1. Fill one row per account in Accounts; add surgeons, referrers and reservoirs on their tabs (link by acronym).</t>
+          <t>0. On the Territory tab, put your name and the states/areas you cover — this is your region.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>1. Fill one row per account in Accounts; add surgeons, referrers and reservoirs on their tabs (link by acronym).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
           <t>2. Run:  python3 build_from_template.py  &lt;thisfile&gt;.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
-    </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>3. Open account-cards.html (or -standalone.html), click “Load my data”, choose the generated .json.</t>
-        </is>
-      </c>
+      <c r="A6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
+          <t>3. Open account-cards.html (or -standalone.html), click “Load my data”, choose the generated .json.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
           <t>4. Everything is editable in the tool; Export saves your edits.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
-    </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Hover any column header for help. Numbers can be left blank (treated as 0).</t>
-        </is>
-      </c>
+      <c r="A9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Reservoir factor_pct blank = indication default (Rad-necrosis 20 · Recurrent GBM 12 · Epilepsy 8 · Mets 3).</t>
+          <t>Hover any column header for help. Numbers can be left blank (treated as 0).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Reservoir factor_pct blank = indication default (Rad-necrosis 20 · Recurrent GBM 12 · Epilepsy 8 · Mets 3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>The physician deep-dive research/pedigree is added centrally per territory — see TEAM-ROLLOUT.md.</t>
         </is>
@@ -781,6 +829,87 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>rep_name</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>territory_name</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>states_covered</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>areas_detail</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>region_avg_case</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Your Name</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Northeast</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>NY;NJ;CT;MA</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>NY = NYC metro + Westchester + Long Island</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>18300</v>
+      </c>
+      <c r="F2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1045,7 +1174,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1249,7 +1378,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1332,7 +1461,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>